<commit_message>
move functions to separate file and source
</commit_message>
<xml_diff>
--- a/Europe_freshwater_summary.xlsx
+++ b/Europe_freshwater_summary.xlsx
@@ -640,7 +640,7 @@
       </c>
       <c r="F9"/>
       <c r="G9" t="n">
-        <v>845</v>
+        <v>844587</v>
       </c>
       <c r="H9" t="n">
         <v>841000</v>
@@ -662,7 +662,7 @@
       </c>
       <c r="F10"/>
       <c r="G10" t="n">
-        <v>536</v>
+        <v>536385</v>
       </c>
       <c r="H10" t="n">
         <v>538347</v>
@@ -684,7 +684,7 @@
       </c>
       <c r="F11"/>
       <c r="G11" t="n">
-        <v>1401</v>
+        <v>1401185</v>
       </c>
       <c r="H11" t="n">
         <v>1394030</v>
@@ -706,7 +706,7 @@
       </c>
       <c r="F12"/>
       <c r="G12" t="n">
-        <v>1446</v>
+        <v>1446425</v>
       </c>
       <c r="H12" t="n">
         <v>1447320</v>
@@ -728,7 +728,7 @@
       </c>
       <c r="F13"/>
       <c r="G13" t="n">
-        <v>1741</v>
+        <v>1740569</v>
       </c>
       <c r="H13" t="n">
         <v>1739960</v>
@@ -750,7 +750,7 @@
       </c>
       <c r="F14"/>
       <c r="G14" t="n">
-        <v>1823</v>
+        <v>1822632</v>
       </c>
       <c r="H14" t="n">
         <v>1832170</v>
@@ -2122,7 +2122,7 @@
         <v>13482128</v>
       </c>
       <c r="G78" t="n">
-        <v>6769</v>
+        <v>6769454</v>
       </c>
       <c r="H78" t="n">
         <v>5378000</v>
@@ -2148,7 +2148,7 @@
         <v>14195156</v>
       </c>
       <c r="G79" t="n">
-        <v>7075</v>
+        <v>7075467</v>
       </c>
       <c r="H79" t="n">
         <v>5727432</v>
@@ -2174,7 +2174,7 @@
         <v>12407013</v>
       </c>
       <c r="G80" t="n">
-        <v>6049</v>
+        <v>6049078</v>
       </c>
       <c r="H80" t="n">
         <v>4677074</v>
@@ -2200,7 +2200,7 @@
         <v>18387733</v>
       </c>
       <c r="G81" t="n">
-        <v>9205</v>
+        <v>9204773</v>
       </c>
       <c r="H81" t="n">
         <v>7547190</v>
@@ -2226,7 +2226,7 @@
         <v>21216949</v>
       </c>
       <c r="G82" t="n">
-        <v>10606</v>
+        <v>10606049</v>
       </c>
       <c r="H82" t="n">
         <v>8769907</v>
@@ -2252,7 +2252,7 @@
         <v>26987699</v>
       </c>
       <c r="G83" t="n">
-        <v>13417</v>
+        <v>13416768</v>
       </c>
       <c r="H83" t="n">
         <v>11394220</v>
@@ -2296,7 +2296,7 @@
         <v>77509990</v>
       </c>
       <c r="G85" t="n">
-        <v>38538</v>
+        <v>38538333</v>
       </c>
       <c r="H85" t="n">
         <v>38467000</v>
@@ -2322,7 +2322,7 @@
         <v>71970677</v>
       </c>
       <c r="G86" t="n">
-        <v>35920</v>
+        <v>35920179</v>
       </c>
       <c r="H86" t="n">
         <v>35674249</v>
@@ -2348,7 +2348,7 @@
         <v>69683775</v>
       </c>
       <c r="G87" t="n">
-        <v>35733</v>
+        <v>35732770</v>
       </c>
       <c r="H87" t="n">
         <v>41005875</v>
@@ -2374,7 +2374,7 @@
         <v>77541214</v>
       </c>
       <c r="G88" t="n">
-        <v>38484</v>
+        <v>38483582</v>
       </c>
       <c r="H88" t="n">
         <v>38258905</v>
@@ -2400,7 +2400,7 @@
         <v>106604291</v>
       </c>
       <c r="G89" t="n">
-        <v>54304</v>
+        <v>54304484</v>
       </c>
       <c r="H89" t="n">
         <v>53006770</v>
@@ -2426,7 +2426,7 @@
         <v>118746186</v>
       </c>
       <c r="G90" t="n">
-        <v>61035</v>
+        <v>61035487</v>
       </c>
       <c r="H90" t="n">
         <v>58819110</v>
@@ -3064,7 +3064,7 @@
         <v>59374000</v>
       </c>
       <c r="G121" t="n">
-        <v>32469</v>
+        <v>32469483</v>
       </c>
       <c r="H121" t="n">
         <v>26527000</v>
@@ -3090,7 +3090,7 @@
         <v>0</v>
       </c>
       <c r="G122" t="n">
-        <v>29342</v>
+        <v>29342385</v>
       </c>
       <c r="H122" t="n">
         <v>27519909</v>
@@ -3116,7 +3116,7 @@
         <v>0</v>
       </c>
       <c r="G123" t="n">
-        <v>27390</v>
+        <v>27390265</v>
       </c>
       <c r="H123" t="n">
         <v>26467883</v>
@@ -3142,7 +3142,7 @@
         <v>0</v>
       </c>
       <c r="G124" t="n">
-        <v>26570</v>
+        <v>26569863</v>
       </c>
       <c r="H124" t="n">
         <v>23425000</v>
@@ -3168,7 +3168,7 @@
         <v>0</v>
       </c>
       <c r="G125" t="n">
-        <v>25609</v>
+        <v>25608541</v>
       </c>
       <c r="H125" t="n">
         <v>29900800</v>
@@ -3194,7 +3194,7 @@
         <v>0</v>
       </c>
       <c r="G126" t="n">
-        <v>33674</v>
+        <v>33673961</v>
       </c>
       <c r="H126" t="n">
         <v>6651310</v>
@@ -3628,7 +3628,7 @@
         <v>67115389</v>
       </c>
       <c r="G147" t="n">
-        <v>30721</v>
+        <v>30720828</v>
       </c>
       <c r="H147" t="n">
         <v>24954000</v>
@@ -3654,7 +3654,7 @@
         <v>74968917</v>
       </c>
       <c r="G148" t="n">
-        <v>31755</v>
+        <v>31754832</v>
       </c>
       <c r="H148" t="n">
         <v>27861042</v>
@@ -3680,7 +3680,7 @@
         <v>77975735</v>
       </c>
       <c r="G149" t="n">
-        <v>39470</v>
+        <v>39470089</v>
       </c>
       <c r="H149" t="n">
         <v>27893432</v>
@@ -3706,7 +3706,7 @@
         <v>71720005</v>
       </c>
       <c r="G150" t="n">
-        <v>36588</v>
+        <v>36587679</v>
       </c>
       <c r="H150" t="n">
         <v>24696739</v>
@@ -3732,7 +3732,7 @@
         <v>82403423</v>
       </c>
       <c r="G151" t="n">
-        <v>36066</v>
+        <v>36065959</v>
       </c>
       <c r="H151" t="n">
         <v>24820229</v>
@@ -3758,7 +3758,7 @@
         <v>95955284</v>
       </c>
       <c r="G152" t="n">
-        <v>37294</v>
+        <v>37294481</v>
       </c>
       <c r="H152" t="n">
         <v>26587640</v>

</xml_diff>